<commit_message>
Update 9 units in THE HENLEY III 3B tower to 3.5% base discount + AVD stamp duty subsidy scheme
</commit_message>
<xml_diff>
--- a/files/九龙-启德-The Henley III.xlsx
+++ b/files/九龙-启德-The Henley III.xlsx
@@ -19751,18 +19751,18 @@
       </c>
       <c r="J300" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K300" s="5" t="n">
-        <v>21008400</v>
+        <v>24723300</v>
       </c>
       <c r="L300" s="5" t="n">
-        <v>27003</v>
+        <v>31778</v>
       </c>
       <c r="M300" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N300" s="3" t="inlineStr">
@@ -20123,18 +20123,18 @@
       </c>
       <c r="J306" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K306" s="5" t="n">
-        <v>20946080</v>
+        <v>24649960</v>
       </c>
       <c r="L306" s="5" t="n">
-        <v>26923</v>
+        <v>31684</v>
       </c>
       <c r="M306" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N306" s="3" t="inlineStr">
@@ -20495,18 +20495,18 @@
       </c>
       <c r="J312" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K312" s="5" t="n">
-        <v>20882940</v>
+        <v>24575655</v>
       </c>
       <c r="L312" s="5" t="n">
-        <v>26842</v>
+        <v>31588</v>
       </c>
       <c r="M312" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N312" s="3" t="inlineStr">
@@ -20805,18 +20805,18 @@
       </c>
       <c r="J317" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="K317" s="5" t="n">
-        <v>14887920</v>
+        <v>17520540</v>
       </c>
       <c r="L317" s="5" t="n">
-        <v>27570</v>
+        <v>32445</v>
       </c>
       <c r="M317" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N317" s="3" t="inlineStr">
@@ -20867,18 +20867,18 @@
       </c>
       <c r="J318" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K318" s="5" t="n">
-        <v>20819800</v>
+        <v>24501350</v>
       </c>
       <c r="L318" s="5" t="n">
-        <v>26761</v>
+        <v>31493</v>
       </c>
       <c r="M318" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N318" s="3" t="inlineStr">
@@ -21549,18 +21549,18 @@
       </c>
       <c r="J329" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="K329" s="5" t="n">
-        <v>14842820</v>
+        <v>17467465</v>
       </c>
       <c r="L329" s="5" t="n">
-        <v>27487</v>
+        <v>32347</v>
       </c>
       <c r="M329" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N329" s="3" t="inlineStr">
@@ -21611,18 +21611,18 @@
       </c>
       <c r="J330" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K330" s="5" t="n">
-        <v>20756660</v>
+        <v>24427045</v>
       </c>
       <c r="L330" s="5" t="n">
-        <v>26680</v>
+        <v>31397</v>
       </c>
       <c r="M330" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N330" s="3" t="inlineStr">
@@ -22665,18 +22665,18 @@
       </c>
       <c r="J347" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="K347" s="5" t="n">
-        <v>14708340</v>
+        <v>17309205</v>
       </c>
       <c r="L347" s="5" t="n">
-        <v>27238</v>
+        <v>32054</v>
       </c>
       <c r="M347" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N347" s="3" t="inlineStr">
@@ -23037,18 +23037,18 @@
       </c>
       <c r="J353" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="K353" s="5" t="n">
-        <v>14663240</v>
+        <v>17256130</v>
       </c>
       <c r="L353" s="5" t="n">
-        <v>27154</v>
+        <v>31956</v>
       </c>
       <c r="M353" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N353" s="3" t="inlineStr">

</xml_diff>